<commit_message>
feat: 인벤토리 탭 칸을 50으로 줄이고 창고 탭 칸 WarehouseCapacity 50을 둔다 (T-107)
</commit_message>
<xml_diff>
--- a/GameDesign/Excel/Constants.xlsx
+++ b/GameDesign/Excel/Constants.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -618,11 +618,11 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>창고 탭마다 칸 수(자원·캐릭터·장비 각각)</t>
+          <t>인벤토리 탭마다 칸 수(자원·캐릭터·장비 각각)</t>
         </is>
       </c>
     </row>
@@ -630,15 +630,15 @@
       <c r="A11" s="1" t="n"/>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>MailboxCapacity</t>
+          <t>WarehouseCapacity</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>안 받은 우편 상한 — 넘침 보관이 멈추는 선</t>
+          <t>창고 탭마다 칸 수(자원·캐릭터·장비 각각) — 클라는 한 줄 5칸 × 10줄로 그린다</t>
         </is>
       </c>
     </row>
@@ -646,15 +646,15 @@
       <c r="A12" s="1" t="n"/>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>BoxOpenMax</t>
+          <t>MailboxCapacity</t>
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>상자를 한 번에 여는 수</t>
+          <t>안 받은 우편 상한 — 넘침 보관이 멈추는 선</t>
         </is>
       </c>
     </row>
@@ -662,15 +662,15 @@
       <c r="A13" s="1" t="n"/>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>GachaDrawSingle</t>
+          <t>BoxOpenMax</t>
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>뽑기 단차 횟수</t>
+          <t>상자를 한 번에 여는 수</t>
         </is>
       </c>
     </row>
@@ -678,15 +678,15 @@
       <c r="A14" s="1" t="n"/>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>GachaDrawMulti</t>
+          <t>GachaDrawSingle</t>
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>뽑기 연차 횟수</t>
+          <t>뽑기 단차 횟수</t>
         </is>
       </c>
     </row>
@@ -694,15 +694,15 @@
       <c r="A15" s="1" t="n"/>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>SellRatePermille</t>
+          <t>GachaDrawMulti</t>
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>1000</v>
+        <v>10</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>즉시 판매가 = BasePrice × 이 값(천분율) — 거래소 하한과 묶인다</t>
+          <t>뽑기 연차 횟수</t>
         </is>
       </c>
     </row>
@@ -710,15 +710,15 @@
       <c r="A16" s="1" t="n"/>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>AuctionListingHours</t>
+          <t>SellRatePermille</t>
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>48</v>
+        <v>1000</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>거래소·경매장 등록 기간(시간)</t>
+          <t>즉시 판매가 = BasePrice × 이 값(천분율) — 거래소 하한과 묶인다</t>
         </is>
       </c>
     </row>
@@ -726,15 +726,15 @@
       <c r="A17" s="1" t="n"/>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>AuctionMaxActiveListings</t>
+          <t>AuctionListingHours</t>
         </is>
       </c>
       <c r="C17" s="7" t="n">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>1인 판매 중 매물 상한</t>
+          <t>거래소·경매장 등록 기간(시간)</t>
         </is>
       </c>
     </row>
@@ -742,15 +742,15 @@
       <c r="A18" s="1" t="n"/>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>AuctionMaxUnitPrice</t>
+          <t>AuctionMaxActiveListings</t>
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>1000000000000</v>
+        <v>20</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>경매 단가 상한(1조) — 하한은 즉시 판매가. 단가×수량×수수료가 long을 넘지 않게</t>
+          <t>1인 판매 중 매물 상한</t>
         </is>
       </c>
     </row>
@@ -758,15 +758,15 @@
       <c r="A19" s="1" t="n"/>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>AuctionMaxListingCount</t>
+          <t>AuctionMaxUnitPrice</t>
         </is>
       </c>
       <c r="C19" s="7" t="n">
-        <v>9999</v>
+        <v>1000000000000</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>경매 한 번에 올리는 수량 상한 — 보유량이 더 많아도 여기서 자른다(단가 상한과 한 쌍)</t>
+          <t>경매 단가 상한(1조) — 하한은 즉시 판매가. 단가×수량×수수료가 long을 넘지 않게</t>
         </is>
       </c>
     </row>
@@ -774,15 +774,15 @@
       <c r="A20" s="1" t="n"/>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>AuctionListingFeePermille</t>
+          <t>AuctionMaxListingCount</t>
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>10</v>
+        <v>9999</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>등록비 = 총액 × 이 값(천분율, 최소 1) — 만료면 환급</t>
+          <t>경매 한 번에 올리는 수량 상한 — 보유량이 더 많아도 여기서 자른다(단가 상한과 한 쌍)</t>
         </is>
       </c>
     </row>
@@ -790,15 +790,15 @@
       <c r="A21" s="1" t="n"/>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>AuctionSaleFeePermille</t>
+          <t>AuctionListingFeePermille</t>
         </is>
       </c>
       <c r="C21" s="7" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>판매 수수료 = 판매액 × 이 값(천분율)</t>
+          <t>등록비 = 총액 × 이 값(천분율, 최소 1) — 만료면 환급</t>
         </is>
       </c>
     </row>
@@ -806,15 +806,15 @@
       <c r="A22" s="1" t="n"/>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>AuctionSearchBurst</t>
+          <t>AuctionSaleFeePermille</t>
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>거래소·경매장 조회 순간 허용 횟수</t>
+          <t>판매 수수료 = 판매액 × 이 값(천분율)</t>
         </is>
       </c>
     </row>
@@ -822,15 +822,15 @@
       <c r="A23" s="1" t="n"/>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>AuctionSearchRefillSeconds</t>
+          <t>AuctionSearchBurst</t>
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>조회 1회가 회복되는 간격(초)</t>
+          <t>거래소·경매장 조회 순간 허용 횟수</t>
         </is>
       </c>
     </row>
@@ -838,15 +838,15 @@
       <c r="A24" s="1" t="n"/>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>CheatMaxCharacterCount</t>
+          <t>AuctionSearchRefillSeconds</t>
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>치트 — 한 번에 지급하는 캐릭터 장수 상한</t>
+          <t>조회 1회가 회복되는 간격(초)</t>
         </is>
       </c>
     </row>
@@ -854,15 +854,15 @@
       <c r="A25" s="1" t="n"/>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>CheatMaxSettleJudges</t>
+          <t>CheatMaxCharacterCount</t>
         </is>
       </c>
       <c r="C25" s="7" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>치트 — 정산을 한 번에 앞당기는 판정 횟수 상한</t>
+          <t>치트 — 한 번에 지급하는 캐릭터 장수 상한</t>
         </is>
       </c>
     </row>
@@ -870,15 +870,15 @@
       <c r="A26" s="1" t="n"/>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>DefaultIndustryLevel</t>
+          <t>CheatMaxSettleJudges</t>
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>게임 시작 시 열린 산업 레벨</t>
+          <t>치트 — 정산을 한 번에 앞당기는 판정 횟수 상한</t>
         </is>
       </c>
     </row>
@@ -886,15 +886,15 @@
       <c r="A27" s="1" t="n"/>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>MarketMaxBuyCount</t>
+          <t>DefaultIndustryLevel</t>
         </is>
       </c>
       <c r="C27" s="7" t="n">
-        <v>9999</v>
+        <v>1</v>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>거래소 한 번 구매 수량 상한</t>
+          <t>게임 시작 시 열린 산업 레벨</t>
         </is>
       </c>
     </row>
@@ -902,15 +902,15 @@
       <c r="A28" s="1" t="n"/>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>MarketPriceLevels</t>
+          <t>MarketMaxBuyCount</t>
         </is>
       </c>
       <c r="C28" s="7" t="n">
-        <v>10</v>
+        <v>9999</v>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>거래소 가격대 줄 수</t>
+          <t>거래소 한 번 구매 수량 상한</t>
         </is>
       </c>
     </row>
@@ -918,15 +918,15 @@
       <c r="A29" s="1" t="n"/>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>DefaultCharacterTid</t>
+          <t>MarketPriceLevels</t>
         </is>
       </c>
       <c r="C29" s="7" t="n">
-        <v>1001</v>
+        <v>10</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>신규 유저 시작 캐릭터 — 전 산업 적성 1 이상이어야 한다</t>
+          <t>거래소 가격대 줄 수</t>
         </is>
       </c>
     </row>
@@ -934,15 +934,15 @@
       <c r="A30" s="1" t="n"/>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>WorkSpeedScale</t>
+          <t>DefaultCharacterTid</t>
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>1000</v>
+        <v>1001</v>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>작업속도 1.0배 = 이 값(천분율 단위) — 바꾸면 ‰ 데이터 전부 재해석</t>
+          <t>신규 유저 시작 캐릭터 — 전 산업 적성 1 이상이어야 한다</t>
         </is>
       </c>
     </row>
@@ -950,15 +950,15 @@
       <c r="A31" s="1" t="n"/>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>BaseCycleSeconds</t>
+          <t>WorkSpeedScale</t>
         </is>
       </c>
       <c r="C31" s="7" t="n">
-        <v>30</v>
+        <v>1000</v>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>1.0배 속도의 판정 1회 시간(초)</t>
+          <t>작업속도 1.0배 = 이 값(천분율 단위) — 바꾸면 ‰ 데이터 전부 재해석</t>
         </is>
       </c>
     </row>
@@ -966,13 +966,29 @@
       <c r="A32" s="1" t="n"/>
       <c r="B32" s="6" t="inlineStr">
         <is>
+          <t>BaseCycleSeconds</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>1.0배 속도의 판정 1회 시간(초)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n"/>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
           <t>MinCycleMs</t>
         </is>
       </c>
-      <c r="C32" s="7" t="n">
+      <c r="C33" s="7" t="n">
         <v>1600</v>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>판정 1회 최소 시간(ms) — 연출 한 바퀴(달리기 1초 + 공격 0.6초)를 보장한다. 실효 주기 = max(이 값, 판정 비용 ÷ 속도)</t>
         </is>

</xml_diff>